<commit_message>
AT4-2277 refined the HSUM config generator and compared it with the spreadsheet generated config.
</commit_message>
<xml_diff>
--- a/FPGA_FDAS_config_generator/HPSEL_Layout_Indices.xlsx
+++ b/FPGA_FDAS_config_generator/HPSEL_Layout_Indices.xlsx
@@ -543,13 +543,13 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="n">
         <v>1</v>
@@ -572,19 +572,19 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
         <v>2</v>
@@ -604,16 +604,16 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
@@ -671,28 +671,28 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
         <v>4</v>
       </c>
       <c r="K7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -706,28 +706,28 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J8" t="n">
         <v>5</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -741,7 +741,7 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -750,19 +750,19 @@
         <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
         <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -776,13 +776,13 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" t="n">
         <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="n">
         <v>4</v>
@@ -791,13 +791,13 @@
         <v>4</v>
       </c>
       <c r="I10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" t="n">
         <v>6</v>
       </c>
       <c r="K10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -858,13 +858,13 @@
         <v>4</v>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K12" t="n">
         <v>9</v>
@@ -887,19 +887,19 @@
         <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I13" t="n">
         <v>7</v>
       </c>
       <c r="J13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K13" t="n">
         <v>10</v>
@@ -919,16 +919,16 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" t="n">
         <v>5</v>
       </c>
       <c r="H14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I14" t="n">
         <v>8</v>
@@ -986,28 +986,28 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>5</v>
       </c>
       <c r="G16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H16" t="n">
         <v>8</v>
       </c>
       <c r="I16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J16" t="n">
         <v>11</v>
       </c>
       <c r="K16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -1021,28 +1021,28 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>5</v>
       </c>
       <c r="G17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H17" t="n">
         <v>8</v>
       </c>
-      <c r="H17" t="n">
-        <v>9</v>
-      </c>
       <c r="I17" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J17" t="n">
         <v>12</v>
       </c>
       <c r="K17" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
@@ -1056,7 +1056,7 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
         <v>4</v>
@@ -1065,19 +1065,19 @@
         <v>5</v>
       </c>
       <c r="G18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H18" t="n">
         <v>9</v>
       </c>
       <c r="I18" t="n">
+        <v>11</v>
+      </c>
+      <c r="J18" t="n">
         <v>12</v>
       </c>
-      <c r="J18" t="n">
-        <v>13</v>
-      </c>
       <c r="K18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
@@ -1091,13 +1091,13 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
         <v>4</v>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G19" t="n">
         <v>8</v>
@@ -1106,13 +1106,13 @@
         <v>9</v>
       </c>
       <c r="I19" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J19" t="n">
         <v>13</v>
       </c>
       <c r="K19" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -1173,13 +1173,13 @@
         <v>8</v>
       </c>
       <c r="H21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I21" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J21" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="K21" t="n">
         <v>17</v>
@@ -1202,19 +1202,19 @@
         <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H22" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I22" t="n">
         <v>13</v>
       </c>
       <c r="J22" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K22" t="n">
         <v>18</v>
@@ -1234,16 +1234,16 @@
         <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G23" t="n">
         <v>9</v>
       </c>
       <c r="H23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I23" t="n">
         <v>14</v>
@@ -1301,28 +1301,28 @@
         <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F25" t="n">
         <v>8</v>
       </c>
       <c r="G25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H25" t="n">
         <v>13</v>
       </c>
       <c r="I25" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J25" t="n">
         <v>18</v>
       </c>
       <c r="K25" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26">
@@ -1336,28 +1336,28 @@
         <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
         <v>8</v>
       </c>
       <c r="G26" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H26" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I26" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J26" t="n">
         <v>19</v>
       </c>
       <c r="K26" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27">
@@ -1371,7 +1371,7 @@
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n">
         <v>6</v>
@@ -1380,19 +1380,19 @@
         <v>8</v>
       </c>
       <c r="G27" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H27" t="n">
         <v>14</v>
       </c>
       <c r="I27" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J27" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K27" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28">
@@ -1406,13 +1406,13 @@
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
         <v>6</v>
       </c>
       <c r="F28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G28" t="n">
         <v>12</v>
@@ -1421,13 +1421,13 @@
         <v>14</v>
       </c>
       <c r="I28" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J28" t="n">
         <v>20</v>
       </c>
       <c r="K28" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29">
@@ -1488,13 +1488,13 @@
         <v>12</v>
       </c>
       <c r="H30" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I30" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J30" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K30" t="n">
         <v>25</v>
@@ -1517,19 +1517,19 @@
         <v>6</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G31" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" t="n">
         <v>19</v>
       </c>
       <c r="J31" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="K31" t="n">
         <v>26</v>
@@ -1549,16 +1549,16 @@
         <v>3</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G32" t="n">
         <v>13</v>
       </c>
       <c r="H32" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I32" t="n">
         <v>20</v>
@@ -1616,28 +1616,28 @@
         <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
         <v>11</v>
       </c>
       <c r="G34" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H34" t="n">
         <v>18</v>
       </c>
       <c r="I34" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J34" t="n">
         <v>25</v>
       </c>
       <c r="K34" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="35">
@@ -1651,28 +1651,28 @@
         <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
         <v>11</v>
       </c>
       <c r="G35" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H35" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I35" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J35" t="n">
         <v>26</v>
       </c>
       <c r="K35" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="36">
@@ -1686,7 +1686,7 @@
         <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
         <v>8</v>
@@ -1695,19 +1695,19 @@
         <v>11</v>
       </c>
       <c r="G36" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H36" t="n">
         <v>19</v>
       </c>
       <c r="I36" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J36" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K36" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37">
@@ -1721,13 +1721,13 @@
         <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
         <v>8</v>
       </c>
       <c r="F37" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G37" t="n">
         <v>16</v>
@@ -1736,13 +1736,13 @@
         <v>19</v>
       </c>
       <c r="I37" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J37" t="n">
         <v>27</v>
       </c>
       <c r="K37" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38">
@@ -1803,13 +1803,13 @@
         <v>16</v>
       </c>
       <c r="H39" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I39" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J39" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K39" t="n">
         <v>33</v>
@@ -1832,19 +1832,19 @@
         <v>8</v>
       </c>
       <c r="F40" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G40" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H40" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I40" t="n">
         <v>25</v>
       </c>
       <c r="J40" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K40" t="n">
         <v>34</v>
@@ -1864,16 +1864,16 @@
         <v>4</v>
       </c>
       <c r="E41" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F41" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G41" t="n">
         <v>17</v>
       </c>
       <c r="H41" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I41" t="n">
         <v>26</v>
@@ -1931,28 +1931,28 @@
         <v>5</v>
       </c>
       <c r="D43" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
         <v>14</v>
       </c>
       <c r="G43" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H43" t="n">
         <v>23</v>
       </c>
       <c r="I43" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J43" t="n">
         <v>32</v>
       </c>
       <c r="K43" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="44">
@@ -1966,28 +1966,28 @@
         <v>5</v>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E44" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F44" t="n">
         <v>14</v>
       </c>
       <c r="G44" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H44" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I44" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J44" t="n">
         <v>33</v>
       </c>
       <c r="K44" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="45">
@@ -2001,7 +2001,7 @@
         <v>5</v>
       </c>
       <c r="D45" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E45" t="n">
         <v>10</v>
@@ -2010,19 +2010,19 @@
         <v>14</v>
       </c>
       <c r="G45" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H45" t="n">
         <v>24</v>
       </c>
       <c r="I45" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J45" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K45" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="46">
@@ -2036,13 +2036,13 @@
         <v>5</v>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E46" t="n">
         <v>10</v>
       </c>
       <c r="F46" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G46" t="n">
         <v>20</v>
@@ -2051,13 +2051,13 @@
         <v>24</v>
       </c>
       <c r="I46" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J46" t="n">
         <v>34</v>
       </c>
       <c r="K46" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47">
@@ -2091,7 +2091,9 @@
       <c r="J47" t="n">
         <v>35</v>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2113,10 +2115,10 @@
         <v>15</v>
       </c>
       <c r="G48" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H48" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I48" t="n">
         <v>31</v>
@@ -2124,7 +2126,9 @@
       <c r="J48" t="n">
         <v>36</v>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2140,10 +2144,10 @@
         <v>5</v>
       </c>
       <c r="E49" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F49" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G49" t="n">
         <v>21</v>
@@ -2157,7 +2161,9 @@
       <c r="J49" t="n">
         <v>37</v>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2203,22 +2209,22 @@
         <v>6</v>
       </c>
       <c r="D51" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E51" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F51" t="n">
         <v>17</v>
       </c>
       <c r="G51" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H51" t="n">
         <v>28</v>
       </c>
       <c r="I51" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J51" t="n">
         <v>39</v>
@@ -2236,22 +2242,22 @@
         <v>6</v>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E52" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F52" t="n">
         <v>17</v>
       </c>
       <c r="G52" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H52" t="n">
         <v>29</v>
       </c>
       <c r="I52" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J52" t="n">
         <v>40</v>
@@ -2269,22 +2275,22 @@
         <v>6</v>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E53" t="n">
         <v>12</v>
       </c>
       <c r="F53" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G53" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H53" t="n">
         <v>29</v>
       </c>
       <c r="I53" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J53" t="n">
         <v>41</v>
@@ -2319,7 +2325,9 @@
       <c r="I54" t="n">
         <v>36</v>
       </c>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="n">
+        <v>42</v>
+      </c>
       <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
@@ -2342,10 +2350,10 @@
         <v>18</v>
       </c>
       <c r="G55" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H55" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I55" t="n">
         <v>37</v>
@@ -2367,10 +2375,10 @@
         <v>6</v>
       </c>
       <c r="E56" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F56" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G56" t="n">
         <v>25</v>
@@ -2426,22 +2434,22 @@
         <v>7</v>
       </c>
       <c r="D58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F58" t="n">
         <v>20</v>
       </c>
       <c r="G58" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H58" t="n">
         <v>33</v>
       </c>
       <c r="I58" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
@@ -2457,22 +2465,22 @@
         <v>7</v>
       </c>
       <c r="D59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E59" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F59" t="n">
         <v>20</v>
       </c>
       <c r="G59" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H59" t="n">
         <v>34</v>
       </c>
       <c r="I59" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
@@ -2488,22 +2496,22 @@
         <v>7</v>
       </c>
       <c r="D60" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E60" t="n">
         <v>14</v>
       </c>
       <c r="F60" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G60" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H60" t="n">
         <v>34</v>
       </c>
       <c r="I60" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
@@ -2533,7 +2541,9 @@
       <c r="H61" t="n">
         <v>35</v>
       </c>
-      <c r="I61" t="inlineStr"/>
+      <c r="I61" t="n">
+        <v>42</v>
+      </c>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
     </row>
@@ -2554,7 +2564,7 @@
         <v>14</v>
       </c>
       <c r="F62" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G62" t="n">
         <v>29</v>
@@ -2606,16 +2616,16 @@
         <v>8</v>
       </c>
       <c r="D64" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E64" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F64" t="n">
         <v>23</v>
       </c>
       <c r="G64" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H64" t="n">
         <v>38</v>
@@ -2635,7 +2645,7 @@
         <v>8</v>
       </c>
       <c r="D65" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E65" t="n">
         <v>16</v>
@@ -2644,7 +2654,7 @@
         <v>23</v>
       </c>
       <c r="G65" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H65" t="n">
         <v>39</v>
@@ -2675,7 +2685,9 @@
       <c r="G66" t="n">
         <v>32</v>
       </c>
-      <c r="H66" t="inlineStr"/>
+      <c r="H66" t="n">
+        <v>40</v>
+      </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
@@ -2697,12 +2709,14 @@
         <v>16</v>
       </c>
       <c r="F67" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G67" t="n">
         <v>33</v>
       </c>
-      <c r="H67" t="inlineStr"/>
+      <c r="H67" t="n">
+        <v>41</v>
+      </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
@@ -2729,7 +2743,9 @@
       <c r="G68" t="n">
         <v>34</v>
       </c>
-      <c r="H68" t="inlineStr"/>
+      <c r="H68" t="n">
+        <v>42</v>
+      </c>
       <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
@@ -2745,16 +2761,16 @@
         <v>9</v>
       </c>
       <c r="D69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E69" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F69" t="n">
         <v>26</v>
       </c>
       <c r="G69" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
@@ -2772,7 +2788,7 @@
         <v>9</v>
       </c>
       <c r="D70" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E70" t="n">
         <v>18</v>
@@ -2781,7 +2797,7 @@
         <v>26</v>
       </c>
       <c r="G70" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
@@ -2832,7 +2848,7 @@
         <v>18</v>
       </c>
       <c r="F72" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G72" t="n">
         <v>37</v>
@@ -2880,16 +2896,16 @@
         <v>10</v>
       </c>
       <c r="D74" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F74" t="n">
         <v>29</v>
       </c>
       <c r="G74" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr"/>
@@ -2907,7 +2923,7 @@
         <v>10</v>
       </c>
       <c r="D75" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E75" t="n">
         <v>20</v>
@@ -2916,7 +2932,7 @@
         <v>29</v>
       </c>
       <c r="G75" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
@@ -2942,7 +2958,9 @@
       <c r="F76" t="n">
         <v>30</v>
       </c>
-      <c r="G76" t="inlineStr"/>
+      <c r="G76" t="n">
+        <v>40</v>
+      </c>
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
@@ -2962,12 +2980,14 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F77" t="n">
         <v>31</v>
       </c>
-      <c r="G77" t="inlineStr"/>
+      <c r="G77" t="n">
+        <v>41</v>
+      </c>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr"/>
@@ -2987,12 +3007,14 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F78" t="n">
-        <v>32</v>
-      </c>
-      <c r="G78" t="inlineStr"/>
+        <v>31</v>
+      </c>
+      <c r="G78" t="n">
+        <v>42</v>
+      </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
@@ -3006,18 +3028,20 @@
         <v>1</v>
       </c>
       <c r="C79" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D79" t="n">
         <v>11</v>
       </c>
       <c r="E79" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F79" t="n">
-        <v>33</v>
-      </c>
-      <c r="G79" t="inlineStr"/>
+        <v>32</v>
+      </c>
+      <c r="G79" t="n">
+        <v>42</v>
+      </c>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
@@ -3031,16 +3055,16 @@
         <v>2</v>
       </c>
       <c r="C80" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D80" t="n">
         <v>11</v>
       </c>
       <c r="E80" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F80" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr"/>
@@ -3062,10 +3086,10 @@
         <v>11</v>
       </c>
       <c r="E81" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F81" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
@@ -3081,16 +3105,16 @@
         <v>4</v>
       </c>
       <c r="C82" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D82" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E82" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F82" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
@@ -3106,16 +3130,16 @@
         <v>5</v>
       </c>
       <c r="C83" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D83" t="n">
         <v>12</v>
       </c>
       <c r="E83" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F83" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
@@ -3137,10 +3161,10 @@
         <v>12</v>
       </c>
       <c r="E84" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F84" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr"/>
@@ -3156,16 +3180,16 @@
         <v>7</v>
       </c>
       <c r="C85" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D85" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E85" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F85" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr"/>
@@ -3181,16 +3205,16 @@
         <v>8</v>
       </c>
       <c r="C86" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D86" t="n">
         <v>13</v>
       </c>
       <c r="E86" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F86" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
@@ -3212,10 +3236,10 @@
         <v>13</v>
       </c>
       <c r="E87" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F87" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr"/>
@@ -3231,15 +3255,17 @@
         <v>10</v>
       </c>
       <c r="C88" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D88" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E88" t="n">
-        <v>28</v>
-      </c>
-      <c r="F88" t="inlineStr"/>
+        <v>27</v>
+      </c>
+      <c r="F88" t="n">
+        <v>40</v>
+      </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
@@ -3254,15 +3280,17 @@
         <v>11</v>
       </c>
       <c r="C89" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D89" t="n">
         <v>14</v>
       </c>
       <c r="E89" t="n">
-        <v>29</v>
-      </c>
-      <c r="F89" t="inlineStr"/>
+        <v>27</v>
+      </c>
+      <c r="F89" t="n">
+        <v>41</v>
+      </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
@@ -3283,9 +3311,11 @@
         <v>14</v>
       </c>
       <c r="E90" t="n">
-        <v>30</v>
-      </c>
-      <c r="F90" t="inlineStr"/>
+        <v>28</v>
+      </c>
+      <c r="F90" t="n">
+        <v>42</v>
+      </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="inlineStr"/>
@@ -3300,13 +3330,13 @@
         <v>2</v>
       </c>
       <c r="C91" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D91" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E91" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
@@ -3323,13 +3353,13 @@
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D92" t="n">
         <v>15</v>
       </c>
       <c r="E92" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
@@ -3352,7 +3382,7 @@
         <v>15</v>
       </c>
       <c r="E93" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
@@ -3369,13 +3399,13 @@
         <v>5</v>
       </c>
       <c r="C94" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D94" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E94" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
@@ -3392,13 +3422,13 @@
         <v>6</v>
       </c>
       <c r="C95" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D95" t="n">
         <v>16</v>
       </c>
       <c r="E95" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
@@ -3421,7 +3451,7 @@
         <v>16</v>
       </c>
       <c r="E96" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
@@ -3438,13 +3468,13 @@
         <v>8</v>
       </c>
       <c r="C97" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D97" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E97" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
@@ -3461,13 +3491,13 @@
         <v>9</v>
       </c>
       <c r="C98" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D98" t="n">
         <v>17</v>
       </c>
       <c r="E98" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
@@ -3490,7 +3520,7 @@
         <v>17</v>
       </c>
       <c r="E99" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
@@ -3507,13 +3537,13 @@
         <v>11</v>
       </c>
       <c r="C100" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D100" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E100" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
@@ -3530,13 +3560,13 @@
         <v>1</v>
       </c>
       <c r="C101" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D101" t="n">
         <v>18</v>
       </c>
       <c r="E101" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr"/>
@@ -3559,7 +3589,7 @@
         <v>18</v>
       </c>
       <c r="E102" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
@@ -3576,13 +3606,13 @@
         <v>3</v>
       </c>
       <c r="C103" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D103" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E103" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
@@ -3599,13 +3629,13 @@
         <v>4</v>
       </c>
       <c r="C104" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D104" t="n">
         <v>19</v>
       </c>
       <c r="E104" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
@@ -3628,7 +3658,7 @@
         <v>19</v>
       </c>
       <c r="E105" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
@@ -3645,13 +3675,13 @@
         <v>6</v>
       </c>
       <c r="C106" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D106" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E106" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
@@ -3668,13 +3698,13 @@
         <v>7</v>
       </c>
       <c r="C107" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D107" t="n">
         <v>20</v>
       </c>
       <c r="E107" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr"/>
@@ -3697,7 +3727,7 @@
         <v>20</v>
       </c>
       <c r="E108" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
@@ -3714,12 +3744,14 @@
         <v>9</v>
       </c>
       <c r="C109" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D109" t="n">
-        <v>21</v>
-      </c>
-      <c r="E109" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="E109" t="n">
+        <v>41</v>
+      </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr"/>
@@ -3735,12 +3767,14 @@
         <v>10</v>
       </c>
       <c r="C110" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D110" t="n">
-        <v>22</v>
-      </c>
-      <c r="E110" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="E110" t="n">
+        <v>41</v>
+      </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr"/>
@@ -3756,12 +3790,14 @@
         <v>11</v>
       </c>
       <c r="C111" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D111" t="n">
-        <v>23</v>
-      </c>
-      <c r="E111" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="E111" t="n">
+        <v>42</v>
+      </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
       <c r="H111" t="inlineStr"/>
@@ -3777,10 +3813,10 @@
         <v>1</v>
       </c>
       <c r="C112" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D112" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
@@ -3798,10 +3834,10 @@
         <v>2</v>
       </c>
       <c r="C113" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D113" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
@@ -3819,10 +3855,10 @@
         <v>3</v>
       </c>
       <c r="C114" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
@@ -3840,10 +3876,10 @@
         <v>4</v>
       </c>
       <c r="C115" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D115" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
@@ -3861,10 +3897,10 @@
         <v>5</v>
       </c>
       <c r="C116" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D116" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
@@ -3882,10 +3918,10 @@
         <v>6</v>
       </c>
       <c r="C117" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D117" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
@@ -3903,10 +3939,10 @@
         <v>7</v>
       </c>
       <c r="C118" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D118" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
@@ -3924,10 +3960,10 @@
         <v>8</v>
       </c>
       <c r="C119" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D119" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr"/>
@@ -3945,10 +3981,10 @@
         <v>9</v>
       </c>
       <c r="C120" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D120" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr"/>
@@ -3966,10 +4002,10 @@
         <v>10</v>
       </c>
       <c r="C121" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D121" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr"/>
@@ -3987,10 +4023,10 @@
         <v>11</v>
       </c>
       <c r="C122" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D122" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
@@ -4008,10 +4044,10 @@
         <v>1</v>
       </c>
       <c r="C123" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D123" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
@@ -4029,10 +4065,10 @@
         <v>2</v>
       </c>
       <c r="C124" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D124" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr"/>
@@ -4050,10 +4086,10 @@
         <v>3</v>
       </c>
       <c r="C125" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D125" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr"/>
@@ -4071,10 +4107,10 @@
         <v>4</v>
       </c>
       <c r="C126" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D126" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr"/>
@@ -4092,10 +4128,10 @@
         <v>5</v>
       </c>
       <c r="C127" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D127" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr"/>
@@ -4113,10 +4149,10 @@
         <v>6</v>
       </c>
       <c r="C128" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D128" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr"/>
@@ -4134,10 +4170,10 @@
         <v>7</v>
       </c>
       <c r="C129" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D129" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr"/>
@@ -4155,10 +4191,10 @@
         <v>8</v>
       </c>
       <c r="C130" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D130" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr"/>
@@ -4175,8 +4211,12 @@
       <c r="B131" t="n">
         <v>9</v>
       </c>
-      <c r="C131" t="inlineStr"/>
-      <c r="D131" t="inlineStr"/>
+      <c r="C131" t="n">
+        <v>42</v>
+      </c>
+      <c r="D131" t="n">
+        <v>41</v>
+      </c>
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr"/>
@@ -4192,8 +4232,12 @@
       <c r="B132" t="n">
         <v>10</v>
       </c>
-      <c r="C132" t="inlineStr"/>
-      <c r="D132" t="inlineStr"/>
+      <c r="C132" t="n">
+        <v>42</v>
+      </c>
+      <c r="D132" t="n">
+        <v>42</v>
+      </c>
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr"/>

</xml_diff>